<commit_message>
CAMBIO EN LIMIPEZA DE CODIGOS
</commit_message>
<xml_diff>
--- a/data/dimensions/dim_sexo.xlsx
+++ b/data/dimensions/dim_sexo.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\snies-spadies-etl\data\dimensions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\snies-spadies-etl\data\dimensions\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A27EE1-0F06-40D0-BCDF-8CE3565E2AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>descripcion</t>
   </si>
@@ -35,16 +36,19 @@
     <t>FEMENINO</t>
   </si>
   <si>
-    <t>NO DEFINIDO</t>
-  </si>
-  <si>
     <t>codigo</t>
+  </si>
+  <si>
+    <t>TRANS</t>
+  </si>
+  <si>
+    <t>NO BINARIO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -355,13 +359,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -388,7 +392,15 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>